<commit_message>
Update debates data - 2026-04-28
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -76,6 +76,137 @@
   </si>
   <si>
     <t xml:space="preserve">M. Loïc Dobler est le premier suppléant de la liste 1 Parti socialiste jurassien (PSJ). M. Dobler est chef de service à l'Établissement cantonal des assurances sociales du canton du Jura (ECAS Jura). Le gouvernement de la République et canton du Jura l'a proclamé élu par arrêté du 24 mars 2026. Le bureau a constaté que l'élection de M. Loïc Dobler, né le 7 avril 1987, originaire de Mümliswil-Ramiswil dans le canton de Soleure, domicilié à Glovelier, a été validée. M. Dobler remplace notre ancien collègue Pierre-Alain Fridez. Sur la base des indications communiquées par M. Dobler, le bureau n'a identifié aucune activité incompatible avec l'exercice d'un mandat parlementaire au sens de l'article 144 de la Constitution fédérale et de l'article 14 de la loi sur le Parlement. Il propose dès lors de constater formellement l'élection de M. Loïc Dobler.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373693</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michaud Gigon Sophie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Par cette initiative, le canton du Jura demande que la législation fédérale soit adaptée pour interdire les importations de denrées alimentaires dont les méthodes de production ne respecteraient pas les normes en vigueur en Suisse. On y retrouve l'esprit de l'initiative populaire "Fair-Food" : exiger la même chose des importations que de l'agriculture suisse, plus d'équité et de durabilité. "Fair-Food" voulait mettre de la justice dans nos assiettes. Un bénéfice qui vise les producteurs et l'env</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Par cette initiative, le canton du Jura demande que la législation fédérale soit adaptée pour interdire les importations de denrées alimentaires dont les méthodes de production ne respecteraient pas les normes en vigueur en Suisse. On y retrouve l'esprit de l'initiative populaire "Fair-Food" : exiger la même chose des importations que de l'agriculture suisse, plus d'équité et de durabilité. "Fair-Food" voulait mettre de la justice dans nos assiettes. Un bénéfice qui vise les producteurs et l'environnement à l'étranger, comme les familles de l'agriculture, ici en Suisse. La Suisse romande avait soutenu cette initiative en 2018, alors qu'elle était rejetée au niveau suisse.
+Depuis plusieurs années, un élément prépondérant de la politique étrangère suisse a été la multiplication des accords de libre-échange avec d'autres pays. Prenons par exemple les accords avec l'Indonésie et le Mercosur, pour les plus récents. Il s'agit d'acteurs dont les standards agricoles, que ce soit en matière de protection de l'environnement ou de bien-être animal, ne sont en aucun cas équivalents à ceux en vigueur dans notre pays, malgré certaines provisions prévues dans les accords. Cela a des conséquences non négligeables pour l'agriculture suisse. Moins compétitive, notamment en raison des coûts de production plus élevés, elle est soumise à une concurrence qui peut être déloyale vis-à-vis des produits étrangers lorsque ceux-ci ne respectent pas les mêmes normes. L'initiative du canton du Jura s'est inscrite dans le contexte de la révolte paysanne face à ces revenus et ces conditions de marché, et a été déposée en mars 2024, l'idée centrale étant l'équité économique et la défense de l'agriculture suisse.
+Face à cette situation, il faut reconnaître que les solutions déjà en place ont montré leurs limites. Ainsi, les labels et étiquetages d'aliments stigmatisant certaines pratiques sont moins complets que des règles plus contraignantes s'appliquant à tous les acteurs sur le marché suisse. Si les standards agricoles suisses sont stricts, notamment pour freiner les impacts environnementaux, les standards appliqués par certains pays peuvent causer de véritables dommages, détruisant la biodiversité ou soumettant les travailleuses et les travailleurs à des conditions de travail inacceptables. En autorisant ces importations, la Suisse cautionne ces méthodes. Refuser les denrées agricoles qui ne répondent pas à certains standards, c'est, à notre échelle, prendre nos responsabilités pour une agriculture plus écologique et humaine au niveau mondial. C'est aussi renforcer la protection des agriculteurs et des agricultrices suisses face à une concurrence déloyale.
+Pour ces deux raisons, l'impact à l'étranger comme la concurrence pour l'agriculture suisse, une minorité de votre Commission de l'économie et des redevances vous enjoint à donner suite à cette initiative du canton du Jura.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pamini Paolo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mi esprimo a nome della Commissione dell'economia e dei tributi sull'oggetto 24.326, l'iniziativa cantonale del Canton Giura "Una politica federale 'a deforestazione zero'".
+Die Initiative fordert den Bund auf, das Bundesrecht so anzupassen, dass Rohstoffe und ihre Nebenprodukte, die auf dem Schweizer Markt in Verkehr gebracht werden oder für den Export bestimmt sind, nicht mit Entwaldung in Verbindung stehen.
+Konkret geht es darum, die EU-Verordnung für entwaldungsfreie Produkte (EU Regulation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mi esprimo a nome della Commissione dell'economia e dei tributi sull'oggetto 24.326, l'iniziativa cantonale del Canton Giura "Una politica federale 'a deforestazione zero'".
+Die Initiative fordert den Bund auf, das Bundesrecht so anzupassen, dass Rohstoffe und ihre Nebenprodukte, die auf dem Schweizer Markt in Verkehr gebracht werden oder für den Export bestimmt sind, nicht mit Entwaldung in Verbindung stehen.
+Konkret geht es darum, die EU-Verordnung für entwaldungsfreie Produkte (EU Regulation on Deforestation-free Products - EUDR), ins Schweizer Recht zu übernehmen. Diese verbietet die Vermarktung von Produkten, die mit Entwaldung in Zusammenhang stehen, wie etwa Palmöl, Kakao, Kaffee, Rindfleisch, Kautschuk und Holz. Die Begründung des Kantons Jura ist zweifach. Einerseits sollen Wettbewerbsnachteile für Schweizer Unternehmen vermieden werden, die in die EU exportieren. Andererseits soll ein Beitrag zur globalen Bekämpfung der Entwaldung sowie zum Schutz der Biodiversität geleistet werden.
+La commission, par 16 voix contre 7 et 2 abstentions, vous propose de ne pas donner suite à l'initiative. Les principales motivations sont les suivantes. L'initiative entraînerait une incertitude réglementaire. Vu que l'application du règlement européen a déjà été reportée à plusieurs reprises, procéder dès à présent à une reprise anticipée entraînerait une incertitude quant à sa mise en oeuvre. Il y aurait aussi des problèmes au niveau des charges administratives élevées. La traçabilité de la certification "sans déforestation" impliquerait des coûts significatifs pour les entreprises, en particulier pour les PME. Finalement, l'initiative aurait une portée très large. Il ne s'agirait pas uniquement des produits suisses, mais également des matières premières, importées et transformées dans notre pays, avec des effets systématiques sur des secteurs économiques entiers.
+Une minorité de la commission vous propose en revanche de donner suite à l'initiative. Je pense que ma collègue, Mme la conseillère nationale Sophie Michaud Gigon, va vous en expliquer les motivations.
+Permettetemi tuttavia una considerazione importante che è stata sollevata anche durante i lavori commissionali. 
+Il mondo sta diventando sempre più verde. Ci sono dati satellitari della Nasa, in particolare le serie storiche Modis e precedenti, che mostrano a partire dagli anni Ottanta un continuo inverdimento della terra e un continuo aumento della massa forestale. La letteratura scientifica di alto livello è chiara su questo punto. Non abbiamo un problema di deforestazione e di diminuzione della vegetazione a livello globale. Lo studio intitolato "Greening of the earth and its drivers" pubblicato su "Nature Climate Change" nel 2016 da Zhu e altri coautori, evidenzia che nel periodo dal 1982 al 2009 tra il 25 per cento e il 50 per cento delle superfici vegetate del pianeta mostra un aumento della copertura fogliare, mentre solo una minima parte registra un declino. Lo stesso studio attribuisce circa il 70 per cento di questo inverdimento all'aumento della concentrazione di anidride carbonica, che agisce come fertilizzante, aumentando la fotosintesi. Forse non tutti ne sono coscienti, ma l'anidride carbonica è il miglior fertilizzante delle piante perché è quello che le piante mangiano. 
+Ulteriori studi su riviste come "Nature Sustainability", "Nature Reviews Earth and Environment", nonché "Nature Climate Change" confermano con dati dal 1981 fino al 2020 e paper pubblicati pochi anni fa, che il fenomeno è reale. I fattori principali sono l'aumento di anidride carbonica, la gestione del territorio e i cambiamenti climatici. In altre parole, la CO2 non è solo un fattore climatico, ma è un input fondamentale per la crescita vegetale, perché è il cibo delle piante. La CO2, alla prova dei fatti, è uno dei migliori fertilizzanti. Questo non vuol dire negare il problema della deforestazione, ma va messo in una chiara prospettiva.
+Vor diesem Hintergrund beantragt Ihnen die Kommission, der Initiative keine Folge zu geben. Sie erachtet eine einseitige Übernahme der europäischen Regelung zum jetzigen Zeitpunkt als verfrüht und mit erheblichen Belastungen verbunden.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cette initiative vise à adapter la législation en vigueur pour garantir que les matières premières et produits mis sur le marché suisse ne soient pas issus de la déforestation. Elle vise à lutter contre la déforestation importée. Certains produits, comme le cacao, le soja, le café, la viande bovine ou l'huile de palme, peuvent occasionner à large échelle une déforestation de forêts tropicales. Celles-ci sont pourtant essentielles pour les populations et pays concernés, mais aussi pour l'humanité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cette initiative vise à adapter la législation en vigueur pour garantir que les matières premières et produits mis sur le marché suisse ne soient pas issus de la déforestation. Elle vise à lutter contre la déforestation importée. Certains produits, comme le cacao, le soja, le café, la viande bovine ou l'huile de palme, peuvent occasionner à large échelle une déforestation de forêts tropicales. Celles-ci sont pourtant essentielles pour les populations et pays concernés, mais aussi pour l'humanité comme puits de carbone. Cette initiative du canton du Jura a trait non seulement à la responsabilité des entreprises, mais aussi à la mise en conformité des entreprises suisses aux normes du marché européen.
+Elle s'inscrit en particulier dans le contexte de la mise en oeuvre prochaine du règlement européen sur la déforestation adopté par les instances de l'Union européenne en 2023. Ce règlement prévoit de nouvelles mesures de diligence pour les opérateurs du marché européen utilisant des matières premières telles que cacao, caoutchouc ou bois. Ces nouvelles obligations toucheront principalement les grandes entreprises et consisteront à prouver systématiquement, notamment par la communication de leurs origines géographiques, que les matières premières utilisées ne sont pas issues de la déforestation. Ces dispositions, qui vont plus loin que celles prévues actuellement par le droit suisse, s'appliqueront aussi aux acteurs d'États tiers qui souhaitent exporter vers l'Union européenne. Se pose donc la question fondamentale de la continuité de l'accès au marché européen pour les entreprises suisses. Le Conseil fédéral se repose sur l'absence actuelle de reconnaissance mutuelle pour éviter de devoir adapter les règles en vigueur. Pourtant, l'expérience nous a montré qu'une position attentiste contient des risques non négligeables.
+Nous nous souvenons de la situation de certains secteurs économiques, comme le secteur biomédical, lors de l'arrêt des négociations sur l'accord-cadre avec l'Union européenne. L'absence de reconnaissance mutuelle dans le domaine médical et celui des biotechnologies a fait capoter de nombreux projets et mis en péril des entreprises suisses pourtant florissantes jusqu'alors. La minorité de la Commission de l'économie et des redevances veut éviter qu'une telle situation ne se répète. En entamant dès maintenant le processus législatif en ce sens, nous pourrons disposer d'une base solide lorsque le moment sera venu de négocier une reconnaissance mutuelle avec l'Union européenne. Même de grandes entreprises suisses, qui seraient pourtant les plus touchées par une telle réglementation, s'y sont déclarées favorables. La proactivité est donc de mise pour obtenir à terme une reconnaissance mutuelle et la garantie de l'accès au marché européen.
+Enfin, donner suite à cette initiative ne permettrait pas seulement de faciliter l'accès des entreprises au marché européen, mais aussi de renforcer significativement la protection de l'environnement. La gestion et la diminution de l'impact environnemental de la Suisse en dehors de ses frontières restent aujourd'hui encore le parent pauvre de notre politique environnementale. Reprendre à notre compte les dispositifs mis en place par l'Union européenne nous permettrait de réaliser des progrès significatifs dans ce domaine sans contraintes disproportionnées. Je le rappelle, les forêts primaires représentent une richesse en biodiversité inestimable ainsi que des puits de carbone plus efficaces. Une politique suisse "Zéro déforestation" est donc un pas vers une prise de responsabilité environnementale allant de la production de matières premières à la consommation finale. C'est un engagement de notre pays en faveur du climat et de la biodiversité.
+Ainsi, je vous enjoins, au nom de la minorité de la Commission de l'économie et des redevances, de donner suite à cette initiative du canton du Jura.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373714</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hübscher Martin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Standesinitiative des Kantons Jura wurde am 14. November 2024 eingereicht. Sie verlangt, den Import von Lebensmitteln, deren Herstellung nicht den Schweizer Vorschriften entspricht, zu verbieten. Die Kommission für Wirtschaft und Abgaben des Nationalrates hat an ihrer Sitzung vom 10. Februar 2026 die vom Kanton Jura eingereichte Standesinitiative vorgeprüft. Der Nationalrat ist Zweitrat. Der Ständerat hat der Standesinitiative am 18. Dezember 2025 auf Antrag seiner Kommission mit 32 zu 10 St</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Standesinitiative des Kantons Jura wurde am 14. November 2024 eingereicht. Sie verlangt, den Import von Lebensmitteln, deren Herstellung nicht den Schweizer Vorschriften entspricht, zu verbieten. Die Kommission für Wirtschaft und Abgaben des Nationalrates hat an ihrer Sitzung vom 10. Februar 2026 die vom Kanton Jura eingereichte Standesinitiative vorgeprüft. Der Nationalrat ist Zweitrat. Der Ständerat hat der Standesinitiative am 18. Dezember 2025 auf Antrag seiner Kommission mit 32 zu 10 Stimmen bei 1 Enthaltung keine Folge gegeben. 
+Die Kommissionsmehrheit hält die Forderung der Standesinitiative aus mehreren Gründen für problematisch. Eine Regelung, wonach nur noch nach Schweizer Vorschriften produzierte Lebensmittel importiert werden dürften, stünde nicht nur im Widerspruch zum WTO-Recht, sondern hätte auch eine deutliche Senkung der Versorgung in der Schweiz zur Folge. Verschiedene, auch pflanzliche Produkte wären in der Schweiz kaum in ausreichender Menge verfügbar. Dies würde den Einkaufstourismus verstärken. Zudem wären die Umsetzung und die Kontrolle eines Importverbots sehr schwierig und kaum realisierbar. 
+Auch importierte Lebensmittel müssen dem Schweizer Recht entsprechen; das ist in Artikel 2 des Lebensmittelgesetzes geregelt. Ausgenommen sind jedoch Verfahren und Produktionsmethoden, die sich nicht in den physischen Eigenschaften des Produkts niederschlagen. Deshalb dürfen z. B. Eier aus Batteriehaltung gemäss geltendem Recht importiert werden. Das ist in der Tat ein bisschen störend, aber die Schweiz verfolgt bereits heute eine andere Strategie. Wir setzen auf Deklaration statt auf Verbote. Das hat sich im Grundsatz bewährt. Die Konsumentinnen und Konsumenten haben dadurch die Wahlfreiheit. Neben der Deklaration ist auch die Einführung von Schweizer Nachhaltigkeitsstandards möglich, wie wir das z. B. bei verschiedenen Labels bereits kennen - sei das Bio Suisse, IP-Suisse oder der Branchenstandard Swissmilk Green bei der Milch. Der Weg über die Deklarationspflicht ist richtig. Er ist zwar nicht umfassend, aber er führt indirekt in gewisser Weise auch dazu, dass das Anliegen der Initiative erfüllt werden kann. Das sehen wir beispielsweise beim Kaninchenfleisch oder bei den Eiern.
+Ein komplettes Importverbot von Lebensmitteln, die nicht Schweizer Standards entsprechen, wäre nicht umsetzbar und würde, wie bereits erwähnt, bei etlichen Produkten zu Versorgungslücken führen.
+Eine Kommissionsminderheit will der Standesinitiative Folge geben, um die Bedeutung der Lebensmittelsicherheit und des fairen Wettbewerbs zwischen der Schweizer und der ausländischen Landwirtschaft zu unterstreichen. Beides würde gerade im Zusammenhang mit neuen Handelsabkommen der Schweiz - z. B. mit den USA oder den Mercosur-Staaten - in Zukunft an Aktualität gewinnen.
+Die Kommission beantragt Ihnen mit 15 zu 6 Stimmen bei 3 Enthaltungen, der Standesinitiative keine Folge zu geben. Eine Minderheit beantragt, ihr Folge zu geben. Dieser Antrag wird jetzt gleich durch Frau Michaud Gigon begründet. Herzlichen Dank, wenn Sie der Initiative keine Folge geben.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373721</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pfister Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M-E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es gibt zwei gleichlautende Standesinitiativen aus Basel-Landschaft und Basel-Stadt. Im Kanton Basel-Landschaft ist in der Verfassung verankert, dass sich alle politischen Behörden dafür einzusetzen haben, dass der Kanton Basel-Landschaft zwei Standesstimmen erhalten soll.
+Im Ständerat wurde die Standesinitiative am 16. Juni 2025 ohne Gegenantrag abgelehnt, nachdem die SPK-S einstimmig den Antrag gestellt hatte, ihr keine Folge zu geben. Die SPK Ihres Rates hat die Initiative am 23. Oktober 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es gibt zwei gleichlautende Standesinitiativen aus Basel-Landschaft und Basel-Stadt. Im Kanton Basel-Landschaft ist in der Verfassung verankert, dass sich alle politischen Behörden dafür einzusetzen haben, dass der Kanton Basel-Landschaft zwei Standesstimmen erhalten soll.
+Im Ständerat wurde die Standesinitiative am 16. Juni 2025 ohne Gegenantrag abgelehnt, nachdem die SPK-S einstimmig den Antrag gestellt hatte, ihr keine Folge zu geben. Die SPK Ihres Rates hat die Initiative am 23. Oktober 2025 beraten. Sie hat Kenntnis von der Debatte im Ständerat wie auch von der Diskussion in der SPK-S genommen, in der eine Vertretung des Kantons Basel-Stadt angehört worden war.
+Der Aufbau des Schweizer Staats und die föderalistische Struktur sind das Resultat von Entscheiden in einer geschichtlichen Epoche und der Entwicklung innerhalb der Geschichte. Insofern ist es selbstverständlich absolut legitim, diese historisch gewachsene Ordnung immer wieder darauf hin zu prüfen, ob sie weiter wachsen und anders gestaltet werden soll. Schliesslich hat der neu geschaffene Kanton Jura selbstverständlich zwei Standesstimmen erhalten. Damals wurde den Halbkantonen auf ihr Begehren hin, ebenfalls eine volle Standesstimme zu erhalten, seitens des Bundesrates beschieden, die Totalrevision der Bundesverfassung abzuwarten. Diese Revision schaffte dann zwar den Status der Halbkantone ab, änderte aber nichts daran, dass den historischen Halbkantonen im Ständerat nur je ein Sitz zugestanden wird.
+Insofern ist der Wunsch aus den Kantonen mit einer Standesstimme eine Art Perpetuum mobile der Vergeblichkeit. Beschränkt sich der Wunsch, wie bei dieser Initiative, auf gewisse Kantone wie Basel-Landschaft und Basel-Stadt, wird er mehrheitlich mit dem Argument abgelehnt, wenn schon müsste er für alle Kantone mit einer Standesstimme gelten. Die Minderheitssprecherin aus dem Kanton Basel-Landschaft hat denn auch ein Kommissionspostulat mit diesem Inhalt beantragt. Dieser Antrag wurde mit 15 zu 7 Stimmen bei 1 Enthaltung abgelehnt. Gibt es aber diese Forderung, wird sie abgelehnt, da ihre Annahme faktisch eine Stärkung der eher konservativen, ländlich geprägten Kantone und eine Stärkung der Deutschschweiz gegenüber der Romandie zur Folge hätte, was wiederum das Gleichgewicht in der Schweizer Eidgenossenschaft stören würde.
+Diese beiden Argumente waren dann auch in der SPK Ihres Rates und im Ständerat die zentralen, warum auch diese Standesinitiative abgelehnt wurde. Unabhängig davon, ob man zwei Standesstimmen für eine begrenzte Anzahl von Kantonen oder für alle will, die Mehrheit im Ständerat sowie in der SPK des Nationalrates erachtet es jetzt als nicht opportun, an dieser historisch gewachsenen Ordnung etwas zu ändern - auch in der vermutlich sehr realistischen Erwartung, dass eine solche Änderung keine Mehrheit im Volk, ganz sicher aber nicht bei den Ständen finden würde. Wer das anders sieht, kann mit einer Volksinitiative versuchen, die Probe aufs Exempel zu machen. Das alles ist nicht zynisch gemeint, sondern einfach realpolitisch. Vermutlich sehen alle hier, die von der Bevölkerung aus den Kantonen Basel-Stadt oder Basel-Landschaft gewählt sind, die Sache anders - mit der vollen politischen Legitimität.
+Die Staatspolitische Kommission Ihres Rates beantragt Ihnen mit 18 zu 4 Stimmen bei 1 Enthaltung, der Initiative keine Folge zu geben.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">373725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marti Samira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitte entschuldigen Sie meine Stimmlage. Ich bin etwas erkältet; darum habe ich mir auch erlaubt, einen Becher für den Notfall mitzunehmen. 
+Die vorliegende Standesinitiative des Kantons Basel-Stadt verlangt, wie der Kommissionssprecher ausgeführt hat, dass die beiden Basel zu Kantonen mit vollem Ständerecht aufgewertet werden. Im Namen der Minderheit und auch im Namen der beiden Kantone bitte ich Sie, diese Standesinitiative zu unterstützen und damit dem Grundsatz zuzustimmen, dass das Thema de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitte entschuldigen Sie meine Stimmlage. Ich bin etwas erkältet; darum habe ich mir auch erlaubt, einen Becher für den Notfall mitzunehmen. 
+Die vorliegende Standesinitiative des Kantons Basel-Stadt verlangt, wie der Kommissionssprecher ausgeführt hat, dass die beiden Basel zu Kantonen mit vollem Ständerecht aufgewertet werden. Im Namen der Minderheit und auch im Namen der beiden Kantone bitte ich Sie, diese Standesinitiative zu unterstützen und damit dem Grundsatz zuzustimmen, dass das Thema der Kantone mit halber Standesstimme endlich ernsthaft aufs staatspolitische Tapet gehört. 
+Das Thema beschäftigt unsere Region seit Jahrzehnten. Aufschwung bekam die Debatte aber vor allem auch wieder mit der Gründung des Kantons Jura 1979. Die Eidgenossenschaft entschied damals, nicht zwei Halbkantone, den Kanton Bern und den Kanton Jura, zu gründen und die Standesstimmen zwischen den beiden aufzuteilen, sondern den beiden Kantonen die Gleichbehandlung zu gewähren und zwei Standesstimmen zuzugestehen. Damit wurde damals auch die Zusammensetzung des Ständerates verändert. Anders war es damals bei der Gründung meines Kantons, des Kantons Basel-Landschaft. Die Ländler wehrten sich damals - eine kleine Geschichtsstunde für Sie - erfolgreich gegen die Besetzung durch die Städter. 1832 wurde per Volksabstimmung der Kanton Basel-Landschaft gegründet und dann 1833 nach einem für die Städter verlustreichen Gefecht mit einem entsprechenden Beschluss der Tagsatzung endgültig auch durchgesetzt. Die beiden ehemaligen Halbkantone erhielten dann je eine Stimme im Ständerat. Knapp 150 Jahre später wurde mit der Gründung des Kantons Jura gewissermassen das offizielle Bekenntnis zum Ende der Geschichte der Halbkantone gesetzt. Schon damals monierten die Vertretungen aus dem Kanton Basel-Landschaft, wie es sich denn nun mit ihrem Kanton verhalte, wann sie jetzt endlich gleichbehandelt würden. Der damals zuständige Bundesrat Furgler vertröstete sie, die Frage könne man dann im Rahmen der nächsten Totalrevision der Bundesverfassung diskutieren. Er wolle, sagte er verständlicherweise, jetzt die Gründung des Kantons Jura nicht gefährden. Dann wurden die Halbkantone im Rahmen der Totalrevision zwar abgeschafft und die Gleichheit der Kantone und das Gebot der Gleichbehandlung der Kantone festgehalten, aber das Relikt der sogenannt vollwertigen Kantone mit halber Standesstimme blieb bestehen. 2001 wurde der parlamentarischen Initiative Janiak 01.403, "Basel-Landschaft und Basel-Stadt. Vollberechtigte Kantone", vom Nationalrat ebenfalls keine Folge gegeben. Auch damals wurde dagegen vor allem eingewendet, dass die Verfassung des Kantons Basel-Stadt damals noch das Ziel der Wiedervereinigung beinhaltete. Basel-Land strebte bereits damals die zwei Sitze an, Basel-Stadt aber den Zusammenschluss. Mehr als zehn Jahre später wurde über eine Initiative zur Wiedervereinigung abgestimmt. Basel-Stadt nahm diese an, Basel-Land aber lehnte sie mit über 70 Prozent ab. Unterdessen wurde auch die Verfassung des Kantons Basel-Stadt angepasst. Die Wiedervereinigung ist nun kein offizielles Verfassungsziel mehr, nur die gute Zusammenarbeit. All das zeigt, dass sich seit der Debatte in den 70er-Jahren die Situation auch vor Ort geändert hat und sich beide Kantone als vollwertige und auch selbstständige Kantone verstehen. In der Region wird nicht verstanden, warum man im Unterschied zu praktisch allen anderen Kantonen nur einen Sitz im Ständerat hat und man quasi vom Nachbarkanton Jura, der uns nahe ist und den wir gut kennen, links überholt wurde. 
+Mir ist klar, dass diese Standesinitiative Schwächen hat. Sie klärt nicht, warum neue Ungleichheiten mit den anderen Kantonen mit halber Standesstimme, den Appenzeller Kantonen sowie Nid- und Obwalden, geschaffen werden sollen. Auch das Argument der wirtschaftlichen Stärke, das in der Begründung der Initiative vom Kanton Basel-Stadt genannt wird, überzeugt mich persönlich nicht. Die Standesvertretung soll bekanntlich ja nicht an Wirtschaftsleistung oder an Grösse geknüpft werden. Ich bedauere deshalb - der Kommissionssprecher hat das ebenfalls erwähnt -, dass die Kommission meinen Antrag auf ein Postulat nicht unterstützt hat. Es braucht eine ernsthafte Auslegeordnung zu Reformoptionen, wie die Gleichbehandlung der Regionen bzw. der Kantone unter Berücksichtigung des Gleichgewichts im Bundesstaat erreicht werden können. Das ist keine statische Angelegenheit, die über hundert Jahre genau das gleiche Gleichgewicht darstellt. Sie werden mit mir einverstanden sein, dass die Konfession heute zum Beispiel nicht mehr die entscheidende Konfliktlinie in unserem Bundesstaat ist. Es sind andere Unterschiedlichkeiten, die wir überwinden und über die wir als Bundesstaat zusammenhalten müssen. Es sind sprachliche und kulturelle Differenzen, die es in einem vielfältigen Land wie der Schweiz gibt. Lassen Sie uns darüber nachdenken. Diese Standesinitiative könnte dafür der Anfang sein. 
 </t>
   </si>
 </sst>
@@ -130,8 +261,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I3" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I9"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -516,6 +647,180 @@
         <v>20</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>50</v>
+      </c>
+      <c r="I9" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-04-30
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -228,6 +228,22 @@
 Ich bin für die Demokratie-Initiative, weil ich meinen Mitmenschen auf Augenhöhe begegnen will, nicht, weil ich von ihnen profitiere. Wer mit mir im gleichen Land lebt, soll mitbestimmen können, egal, ob er in Herrliberg oder in Spreitenbach wohnt, egal, ob er Thomas oder Mahmoud heisst, und egal, ob er meiner Meinung ist oder irgendeinen Gugus abstimmt. Ich respektiere nämlich nicht nur Menschen, die ähnlich sind wie ich, sondern alle. 
 Zuletzt noch dies: Wenn Ausländerinnen und Ausländer fünf Jahre lang friedlich sein müssen, um sich den Pass zu verdienen, wie es die Initiative verlangt, könnten wir Schweizerinnen und Schweizer unseren Pass eigentlich abgeben, wenn wir uns innerhalb von fünf Jahren mal menschenverachtend verhalten. Aber dann wäre unsere Demokratie wieder unvollständiger - und dieser Saal um einiges leerer. 
 Ich bitte Sie, die Demokratie-Initiative anzunehmen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">374382</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tuosto Brenda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Suisse romande refuse de payer le prix d'une planification défaillante des CFF et de l'Office fédéral des transports (OFT) pendant une décennie. L'horaire 2025 n'est pas une simple mise à jour technique, c'est un choix politique. Un choix politique de priorisation entre les différentes régions, entre les différentes vitesses, entre transport de voyageurs et transport de marchandises. Il est inadmissible qu'une partie du pays soit contrainte de porter seule le poids de choix politiques de refo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Suisse romande refuse de payer le prix d'une planification défaillante des CFF et de l'Office fédéral des transports (OFT) pendant une décennie. L'horaire 2025 n'est pas une simple mise à jour technique, c'est un choix politique. Un choix politique de priorisation entre les différentes régions, entre les différentes vitesses, entre transport de voyageurs et transport de marchandises. Il est inadmissible qu'une partie du pays soit contrainte de porter seule le poids de choix politiques de refonte de l'horaire. Si les CFF invoquent des problèmes de ponctualité pour justifier ces mesures, ces désagréments ne se justifient absolument pas et ne sauraient être absorbés au seul profit du poumon économique alémanique indûment épargné. En interrompant la liaison IC5 entre Genève et Olten, l'OFT impose aux habitantes et habitants du nord de la Suisse jusqu'à l'ouest du pays une accessibilité au rail dégradée pour la décennie à venir. On ne peut exiger de la Suisse occidentale qu'elle sacrifie sa connectivité pour compenser des retards d'infrastructures qui ne lui incombent pas. L'introduction de l'horaire 2025 marque une régression pour les habitantes et habitants de la ligne du Pied-du-Jura. L'allongement des trajets d'environ 8 pour cent sur toutes les lignes romandes d'importance nationale et la fin des liaisons directes contredisent les objectifs de neutralité carbone de l'Office fédéral de l'environnement. La complexification des parcours est un frein majeur à l'attractivité du rail.
+Le Département fédéral de l'environnement, des transports, de l'énergie et de la communication (DETEC) tente de nous rassurer en parlant de la mise en service du tunnel de Gléresse et de la remise en place du train circulant via le by-pass comme d'une révolution de l'horaire 2030. Restons lucides face à ces éléments de communication qui masquent la réalité du terrain. Le projet de by-pass existait déjà dans Rail 2000. Présenter un simple retour à la normale après travaux comme une avancée stratégique est une lecture un peu trop sélective de la réalité. D'autant plus que l'horaire 2030 ne prévoit aucun rétablissement des correspondances entre la ligne du Pied-du-Jura et celle du Valais, laissant la rupture de charge inchangée à Lausanne. La situation reste donc problématique pour les déplacements de l'Arc jurassien au-delà de Martigny. L'axe du Pied-du-Jura doit être connecté avec des noeuds de correspondance à Zurich, à Bâle et à Lausanne. Les régions d'Argovie, de Soleure, du Jura bernois, du Jura, des deux Bâle, de Neuchâtel et du Nord vaudois doivent rester connectées avec le reste de la Suisse.
+Avec ce postulat, je demande formellement le rétablissement des correspondances entre l'IC5 et l'IR90. Un réseau national n'a de sens que si ses noeuds fonctionnent. Il faut corriger cette erreur de planification maintenant. Le Conseil fédéral nous promet des solutions pour 2030, mais elles sont insuffisantes. Aujourd'hui, l'inertie administrative du DETEC bloque les projets déjà approuvés comme ceux liés à la redondance Lausanne-Genève, à la halte d'Y-Parc ou aux mesures de compensation des 100 millions de francs qui ont été votées ces dernières années et qui pourraient améliorer rapidement la situation. Si nous attendons une nouvelle décision des chambres en 2027 voire 2028, ces études deviendront caduques. Nous allons gaspiller l'argent public en refaisant de nouvelles études déjà payées. Je demande au Conseil fédéral de débloquer ces mesures immédiatement pour sauver ce qui peut l'être.
+En conclusion, nous ne demandons pas de faveur. Nous demandons le respect des engagements pris envers la Suisse occidentale et la Suisse alémanique. L'horaire 2025 est une situation qui, sans intervention politique, deviendra la norme : des liaisons nationales interrompues et des durées de trajet rallongées. Il ne s'agit pas d'exiger des offres ou des investissements supplémentaires, mais simplement de revenir à la normale. La situation d'avant 2025 doit être remise en place totalement et maintenant. Soutenir ce postulat, c'est répondre à l'appel de l'Alliance des villes et des milieux économiques situés sur l'ensemble de l'axe du Pied-du-Jura. La cohésion nationale ne saurait se maintenir si l'on consent à l'isolement d'une grande partie du pays. Je vous remercie pour votre soutien.
 </t>
   </si>
 </sst>
@@ -282,8 +298,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I11"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -871,6 +887,35 @@
         <v>55</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" t="s">
+        <v>58</v>
+      </c>
+      <c r="I11" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>